<commit_message>
Publish catalog 10000_items_cat 1.0.1
</commit_message>
<xml_diff>
--- a/catalog_cloud/catalogos/10000_items_cat.xlsx
+++ b/catalog_cloud/catalogos/10000_items_cat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ventas3\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FB172BC-DA23-43BD-B08B-D492A316359A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D53F37F3-829F-475B-8947-6580CA0D6AFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Código</t>
   </si>
@@ -33,10 +33,19 @@
     <t>Descripción</t>
   </si>
   <si>
-    <t>Referecia_cruzada</t>
-  </si>
-  <si>
     <t>prueba</t>
+  </si>
+  <si>
+    <t>Referecia cruzada</t>
+  </si>
+  <si>
+    <t>prueba2</t>
+  </si>
+  <si>
+    <t>r6666666</t>
+  </si>
+  <si>
+    <t>r7777777</t>
   </si>
 </sst>
 </file>
@@ -354,18 +363,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -373,10 +387,21 @@
         <v>6666666</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>7777777</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>